<commit_message>
remove affinity for outlook false positive
</commit_message>
<xml_diff>
--- a/add-in-ids/add-ins-using-exchange-tokens.xlsx
+++ b/add-in-ids/add-ins-using-exchange-tokens.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28619"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73FFD934-5A53-4CAA-A286-4A76F2C0EACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9BDEF2-8F23-4ECC-BD34-7BD727B64A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4230" yWindow="1035" windowWidth="18180" windowHeight="14130" xr2:uid="{8FF931F1-CAD9-4954-9038-88E82260DB46}"/>
+    <workbookView xWindow="19395" yWindow="465" windowWidth="18180" windowHeight="14130" xr2:uid="{8FF931F1-CAD9-4954-9038-88E82260DB46}"/>
   </bookViews>
   <sheets>
     <sheet name="Add-ins list" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2732" uniqueCount="2622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2729" uniqueCount="2619">
   <si>
     <t>AssetID</t>
   </si>
@@ -3790,15 +3790,6 @@
   </si>
   <si>
     <t>Salesforce Connector</t>
-  </si>
-  <si>
-    <t>wa200002298</t>
-  </si>
-  <si>
-    <t>454185ec-7334-4b9b-96c1-5a32f7462d0e</t>
-  </si>
-  <si>
-    <t>Affinity for Outlook</t>
   </si>
   <si>
     <t>wa200002312</t>
@@ -7981,8 +7972,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}" name="Table1" displayName="Table1" ref="A1:C912" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:C912" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}" name="Table1" displayName="Table1" ref="A1:C911" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:C911" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{39B649A1-0CDF-46AA-A276-6F4F89255D96}" name="AssetID"/>
     <tableColumn id="2" xr3:uid="{C79A1EFF-47FF-488B-A562-E9848648C952}" name="AppId"/>
@@ -8309,7 +8300,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3293B4AA-89CE-4E6A-9112-DA5B905DDA88}">
-  <dimension ref="A1:C912"/>
+  <dimension ref="A1:C911"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
@@ -8323,7 +8314,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2621</v>
+        <v>2618</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -13392,7 +13383,7 @@
       <c r="A463" t="s">
         <v>1283</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B463" s="1" t="s">
         <v>1284</v>
       </c>
       <c r="C463" t="s">
@@ -13403,7 +13394,7 @@
       <c r="A464" t="s">
         <v>1286</v>
       </c>
-      <c r="B464" s="1" t="s">
+      <c r="B464" t="s">
         <v>1287</v>
       </c>
       <c r="C464" t="s">
@@ -13535,7 +13526,7 @@
       <c r="A476" t="s">
         <v>1322</v>
       </c>
-      <c r="B476" t="s">
+      <c r="B476" s="1" t="s">
         <v>1323</v>
       </c>
       <c r="C476" t="s">
@@ -13546,7 +13537,7 @@
       <c r="A477" t="s">
         <v>1325</v>
       </c>
-      <c r="B477" s="1" t="s">
+      <c r="B477" t="s">
         <v>1326</v>
       </c>
       <c r="C477" t="s">
@@ -13577,13 +13568,13 @@
     </row>
     <row r="480" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B480" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="C480" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.25">
@@ -13613,21 +13604,21 @@
         <v>1344</v>
       </c>
       <c r="B483" t="s">
-        <v>1345</v>
+        <v>987</v>
       </c>
       <c r="C483" t="s">
-        <v>1346</v>
+        <v>282</v>
       </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B484" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C484" t="s">
         <v>1347</v>
-      </c>
-      <c r="B484" t="s">
-        <v>987</v>
-      </c>
-      <c r="C484" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
@@ -14210,18 +14201,18 @@
         <v>1505</v>
       </c>
       <c r="C537" t="s">
-        <v>1506</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B538" t="s">
         <v>1507</v>
       </c>
-      <c r="B538" t="s">
+      <c r="C538" t="s">
         <v>1508</v>
-      </c>
-      <c r="C538" t="s">
-        <v>1306</v>
       </c>
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
@@ -14229,18 +14220,18 @@
         <v>1509</v>
       </c>
       <c r="B539" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C539" t="s">
         <v>1510</v>
-      </c>
-      <c r="C539" t="s">
-        <v>1511</v>
       </c>
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B540" t="s">
         <v>1512</v>
-      </c>
-      <c r="B540" t="s">
-        <v>1496</v>
       </c>
       <c r="C540" t="s">
         <v>1513</v>
@@ -14680,18 +14671,18 @@
         <v>1631</v>
       </c>
       <c r="B580" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C580" t="s">
         <v>1632</v>
-      </c>
-      <c r="C580" t="s">
-        <v>1633</v>
       </c>
     </row>
     <row r="581" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A581" t="s">
+        <v>1633</v>
+      </c>
+      <c r="B581" t="s">
         <v>1634</v>
-      </c>
-      <c r="B581" t="s">
-        <v>1496</v>
       </c>
       <c r="C581" t="s">
         <v>1635</v>
@@ -15156,18 +15147,18 @@
         <v>1760</v>
       </c>
       <c r="C623" t="s">
-        <v>1761</v>
+        <v>614</v>
       </c>
     </row>
     <row r="624" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A624" t="s">
+        <v>1761</v>
+      </c>
+      <c r="B624" t="s">
         <v>1762</v>
       </c>
-      <c r="B624" t="s">
+      <c r="C624" t="s">
         <v>1763</v>
-      </c>
-      <c r="C624" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="625" spans="1:3" x14ac:dyDescent="0.25">
@@ -15574,18 +15565,18 @@
         <v>1873</v>
       </c>
       <c r="C661" t="s">
-        <v>1874</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="662" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A662" t="s">
+        <v>1874</v>
+      </c>
+      <c r="B662" t="s">
         <v>1875</v>
       </c>
-      <c r="B662" t="s">
+      <c r="C662" t="s">
         <v>1876</v>
-      </c>
-      <c r="C662" t="s">
-        <v>1189</v>
       </c>
     </row>
     <row r="663" spans="1:3" x14ac:dyDescent="0.25">
@@ -15794,18 +15785,18 @@
         <v>1932</v>
       </c>
       <c r="C681" t="s">
-        <v>1933</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="682" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A682" t="s">
+        <v>1933</v>
+      </c>
+      <c r="B682" t="s">
         <v>1934</v>
       </c>
-      <c r="B682" t="s">
+      <c r="C682" t="s">
         <v>1935</v>
-      </c>
-      <c r="C682" t="s">
-        <v>1389</v>
       </c>
     </row>
     <row r="683" spans="1:3" x14ac:dyDescent="0.25">
@@ -16586,18 +16577,18 @@
         <v>2147</v>
       </c>
       <c r="C753" t="s">
-        <v>2148</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="754" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A754" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B754" t="s">
         <v>2149</v>
       </c>
-      <c r="B754" t="s">
+      <c r="C754" t="s">
         <v>2150</v>
-      </c>
-      <c r="C754" t="s">
-        <v>1337</v>
       </c>
     </row>
     <row r="755" spans="1:3" x14ac:dyDescent="0.25">
@@ -16674,18 +16665,18 @@
         <v>2170</v>
       </c>
       <c r="C761" t="s">
-        <v>2171</v>
+        <v>294</v>
       </c>
     </row>
     <row r="762" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A762" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B762" t="s">
         <v>2172</v>
       </c>
-      <c r="B762" t="s">
+      <c r="C762" t="s">
         <v>2173</v>
-      </c>
-      <c r="C762" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="763" spans="1:3" x14ac:dyDescent="0.25">
@@ -16707,18 +16698,18 @@
         <v>2178</v>
       </c>
       <c r="C764" t="s">
-        <v>2179</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="765" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A765" t="s">
+        <v>2179</v>
+      </c>
+      <c r="B765" t="s">
         <v>2180</v>
       </c>
-      <c r="B765" t="s">
+      <c r="C765" t="s">
         <v>2181</v>
-      </c>
-      <c r="C765" t="s">
-        <v>1522</v>
       </c>
     </row>
     <row r="766" spans="1:3" x14ac:dyDescent="0.25">
@@ -16839,18 +16830,18 @@
         <v>2213</v>
       </c>
       <c r="C776" t="s">
-        <v>2214</v>
+        <v>497</v>
       </c>
     </row>
     <row r="777" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A777" t="s">
+        <v>2214</v>
+      </c>
+      <c r="B777" t="s">
         <v>2215</v>
       </c>
-      <c r="B777" t="s">
+      <c r="C777" t="s">
         <v>2216</v>
-      </c>
-      <c r="C777" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="778" spans="1:3" x14ac:dyDescent="0.25">
@@ -17730,18 +17721,18 @@
         <v>2455</v>
       </c>
       <c r="C857" t="s">
-        <v>2456</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="858" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A858" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B858" t="s">
         <v>2457</v>
       </c>
-      <c r="B858" t="s">
+      <c r="C858" t="s">
         <v>2458</v>
-      </c>
-      <c r="C858" t="s">
-        <v>2441</v>
       </c>
     </row>
     <row r="859" spans="1:3" x14ac:dyDescent="0.25">
@@ -18325,17 +18316,6 @@
       </c>
       <c r="C911" t="s">
         <v>2617</v>
-      </c>
-    </row>
-    <row r="912" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A912" t="s">
-        <v>2618</v>
-      </c>
-      <c r="B912" t="s">
-        <v>2619</v>
-      </c>
-      <c r="C912" t="s">
-        <v>2620</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Exchange token list] remove false positive (#5446)
* remove false positive

* remove affinity for outlook false positive
</commit_message>
<xml_diff>
--- a/add-in-ids/add-ins-using-exchange-tokens.xlsx
+++ b/add-in-ids/add-ins-using-exchange-tokens.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28619"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C71497-A64B-4E37-AA78-608A70459B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9BDEF2-8F23-4ECC-BD34-7BD727B64A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8FF931F1-CAD9-4954-9038-88E82260DB46}"/>
+    <workbookView xWindow="19395" yWindow="465" windowWidth="18180" windowHeight="14130" xr2:uid="{8FF931F1-CAD9-4954-9038-88E82260DB46}"/>
   </bookViews>
   <sheets>
     <sheet name="Add-ins list" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2735" uniqueCount="2625">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2729" uniqueCount="2619">
   <si>
     <t>AssetID</t>
   </si>
@@ -2298,15 +2298,6 @@
     <t>iCIMS Video Studio</t>
   </si>
   <si>
-    <t>wa200000033</t>
-  </si>
-  <si>
-    <t>f762dd1f-92c5-486c-992f-31a61967279d</t>
-  </si>
-  <si>
-    <t>Traction Guest</t>
-  </si>
-  <si>
     <t>wa200000035</t>
   </si>
   <si>
@@ -3799,15 +3790,6 @@
   </si>
   <si>
     <t>Salesforce Connector</t>
-  </si>
-  <si>
-    <t>wa200002298</t>
-  </si>
-  <si>
-    <t>454185ec-7334-4b9b-96c1-5a32f7462d0e</t>
-  </si>
-  <si>
-    <t>Affinity for Outlook</t>
   </si>
   <si>
     <t>wa200002312</t>
@@ -7990,8 +7972,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}" name="Table1" displayName="Table1" ref="A1:C913" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:C913" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}" name="Table1" displayName="Table1" ref="A1:C911" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:C911" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{39B649A1-0CDF-46AA-A276-6F4F89255D96}" name="AssetID"/>
     <tableColumn id="2" xr3:uid="{C79A1EFF-47FF-488B-A562-E9848648C952}" name="AppId"/>
@@ -8318,7 +8300,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3293B4AA-89CE-4E6A-9112-DA5B905DDA88}">
-  <dimension ref="A1:C913"/>
+  <dimension ref="A1:C911"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
@@ -8332,7 +8314,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2624</v>
+        <v>2618</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -11389,15 +11371,15 @@
         <v>830</v>
       </c>
       <c r="B280" t="s">
-        <v>831</v>
+        <v>281</v>
       </c>
       <c r="C280" t="s">
-        <v>832</v>
+        <v>282</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
       <c r="B281" t="s">
         <v>281</v>
@@ -11408,7 +11390,7 @@
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="B282" t="s">
         <v>281</v>
@@ -11419,7 +11401,7 @@
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="B283" t="s">
         <v>281</v>
@@ -11430,7 +11412,7 @@
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="B284" t="s">
         <v>281</v>
@@ -11441,7 +11423,7 @@
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
       <c r="B285" t="s">
         <v>281</v>
@@ -11452,13 +11434,13 @@
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
+        <v>836</v>
+      </c>
+      <c r="B286" t="s">
+        <v>837</v>
+      </c>
+      <c r="C286" t="s">
         <v>838</v>
-      </c>
-      <c r="B286" t="s">
-        <v>281</v>
-      </c>
-      <c r="C286" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
@@ -11477,15 +11459,15 @@
         <v>842</v>
       </c>
       <c r="B288" t="s">
-        <v>843</v>
+        <v>281</v>
       </c>
       <c r="C288" t="s">
-        <v>844</v>
+        <v>282</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>845</v>
+        <v>843</v>
       </c>
       <c r="B289" t="s">
         <v>281</v>
@@ -11496,7 +11478,7 @@
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>846</v>
+        <v>844</v>
       </c>
       <c r="B290" t="s">
         <v>281</v>
@@ -11507,7 +11489,7 @@
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>847</v>
+        <v>845</v>
       </c>
       <c r="B291" t="s">
         <v>281</v>
@@ -11518,13 +11500,13 @@
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
+        <v>846</v>
+      </c>
+      <c r="B292" t="s">
+        <v>847</v>
+      </c>
+      <c r="C292" t="s">
         <v>848</v>
-      </c>
-      <c r="B292" t="s">
-        <v>281</v>
-      </c>
-      <c r="C292" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
@@ -11543,21 +11525,21 @@
         <v>852</v>
       </c>
       <c r="B294" t="s">
-        <v>853</v>
+        <v>281</v>
       </c>
       <c r="C294" t="s">
-        <v>854</v>
+        <v>282</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
+        <v>853</v>
+      </c>
+      <c r="B295" t="s">
+        <v>854</v>
+      </c>
+      <c r="C295" t="s">
         <v>855</v>
-      </c>
-      <c r="B295" t="s">
-        <v>281</v>
-      </c>
-      <c r="C295" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
@@ -11565,15 +11547,15 @@
         <v>856</v>
       </c>
       <c r="B296" t="s">
-        <v>857</v>
+        <v>281</v>
       </c>
       <c r="C296" t="s">
-        <v>858</v>
+        <v>282</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="B297" t="s">
         <v>281</v>
@@ -11584,13 +11566,13 @@
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
+        <v>858</v>
+      </c>
+      <c r="B298" t="s">
+        <v>859</v>
+      </c>
+      <c r="C298" t="s">
         <v>860</v>
-      </c>
-      <c r="B298" t="s">
-        <v>281</v>
-      </c>
-      <c r="C298" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
@@ -11653,21 +11635,21 @@
         <v>876</v>
       </c>
       <c r="B304" t="s">
-        <v>877</v>
+        <v>281</v>
       </c>
       <c r="C304" t="s">
-        <v>878</v>
+        <v>282</v>
       </c>
     </row>
     <row r="305" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
+        <v>877</v>
+      </c>
+      <c r="B305" t="s">
+        <v>878</v>
+      </c>
+      <c r="C305" t="s">
         <v>879</v>
-      </c>
-      <c r="B305" t="s">
-        <v>281</v>
-      </c>
-      <c r="C305" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="306" spans="1:3" x14ac:dyDescent="0.25">
@@ -11675,15 +11657,15 @@
         <v>880</v>
       </c>
       <c r="B306" t="s">
-        <v>881</v>
+        <v>281</v>
       </c>
       <c r="C306" t="s">
-        <v>882</v>
+        <v>282</v>
       </c>
     </row>
     <row r="307" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="B307" t="s">
         <v>281</v>
@@ -11694,7 +11676,7 @@
     </row>
     <row r="308" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="B308" t="s">
         <v>281</v>
@@ -11705,7 +11687,7 @@
     </row>
     <row r="309" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="B309" t="s">
         <v>281</v>
@@ -11716,7 +11698,7 @@
     </row>
     <row r="310" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="B310" t="s">
         <v>281</v>
@@ -11727,7 +11709,7 @@
     </row>
     <row r="311" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="B311" t="s">
         <v>281</v>
@@ -11738,7 +11720,7 @@
     </row>
     <row r="312" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="B312" t="s">
         <v>281</v>
@@ -11749,7 +11731,7 @@
     </row>
     <row r="313" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="B313" t="s">
         <v>281</v>
@@ -11760,7 +11742,7 @@
     </row>
     <row r="314" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="B314" t="s">
         <v>281</v>
@@ -11771,7 +11753,7 @@
     </row>
     <row r="315" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="B315" t="s">
         <v>281</v>
@@ -11782,7 +11764,7 @@
     </row>
     <row r="316" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="B316" t="s">
         <v>281</v>
@@ -11793,7 +11775,7 @@
     </row>
     <row r="317" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="B317" t="s">
         <v>281</v>
@@ -11804,7 +11786,7 @@
     </row>
     <row r="318" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="B318" t="s">
         <v>281</v>
@@ -11815,7 +11797,7 @@
     </row>
     <row r="319" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="B319" t="s">
         <v>281</v>
@@ -11826,7 +11808,7 @@
     </row>
     <row r="320" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="B320" t="s">
         <v>281</v>
@@ -11837,7 +11819,7 @@
     </row>
     <row r="321" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="B321" t="s">
         <v>281</v>
@@ -11848,7 +11830,7 @@
     </row>
     <row r="322" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="B322" t="s">
         <v>281</v>
@@ -11859,7 +11841,7 @@
     </row>
     <row r="323" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="B323" t="s">
         <v>281</v>
@@ -11870,7 +11852,7 @@
     </row>
     <row r="324" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="B324" t="s">
         <v>281</v>
@@ -11881,7 +11863,7 @@
     </row>
     <row r="325" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="B325" t="s">
         <v>281</v>
@@ -11892,7 +11874,7 @@
     </row>
     <row r="326" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="B326" t="s">
         <v>281</v>
@@ -11903,7 +11885,7 @@
     </row>
     <row r="327" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="B327" t="s">
         <v>281</v>
@@ -11914,13 +11896,13 @@
     </row>
     <row r="328" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
+        <v>902</v>
+      </c>
+      <c r="B328" t="s">
+        <v>903</v>
+      </c>
+      <c r="C328" t="s">
         <v>904</v>
-      </c>
-      <c r="B328" t="s">
-        <v>281</v>
-      </c>
-      <c r="C328" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="329" spans="1:3" x14ac:dyDescent="0.25">
@@ -11928,15 +11910,15 @@
         <v>905</v>
       </c>
       <c r="B329" t="s">
-        <v>906</v>
+        <v>281</v>
       </c>
       <c r="C329" t="s">
-        <v>907</v>
+        <v>282</v>
       </c>
     </row>
     <row r="330" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="B330" t="s">
         <v>281</v>
@@ -11947,7 +11929,7 @@
     </row>
     <row r="331" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="B331" t="s">
         <v>281</v>
@@ -11958,7 +11940,7 @@
     </row>
     <row r="332" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="B332" t="s">
         <v>281</v>
@@ -11969,7 +11951,7 @@
     </row>
     <row r="333" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="B333" t="s">
         <v>281</v>
@@ -11980,13 +11962,13 @@
     </row>
     <row r="334" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
+        <v>910</v>
+      </c>
+      <c r="B334" t="s">
+        <v>911</v>
+      </c>
+      <c r="C334" t="s">
         <v>912</v>
-      </c>
-      <c r="B334" t="s">
-        <v>281</v>
-      </c>
-      <c r="C334" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="335" spans="1:3" x14ac:dyDescent="0.25">
@@ -11994,15 +11976,15 @@
         <v>913</v>
       </c>
       <c r="B335" t="s">
-        <v>914</v>
+        <v>281</v>
       </c>
       <c r="C335" t="s">
-        <v>915</v>
+        <v>282</v>
       </c>
     </row>
     <row r="336" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>916</v>
+        <v>914</v>
       </c>
       <c r="B336" t="s">
         <v>281</v>
@@ -12013,13 +11995,13 @@
     </row>
     <row r="337" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
+        <v>915</v>
+      </c>
+      <c r="B337" t="s">
+        <v>916</v>
+      </c>
+      <c r="C337" t="s">
         <v>917</v>
-      </c>
-      <c r="B337" t="s">
-        <v>281</v>
-      </c>
-      <c r="C337" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="338" spans="1:3" x14ac:dyDescent="0.25">
@@ -12052,18 +12034,18 @@
         <v>925</v>
       </c>
       <c r="C340" t="s">
-        <v>926</v>
+        <v>282</v>
       </c>
     </row>
     <row r="341" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
+        <v>926</v>
+      </c>
+      <c r="B341" t="s">
         <v>927</v>
       </c>
-      <c r="B341" t="s">
+      <c r="C341" t="s">
         <v>928</v>
-      </c>
-      <c r="C341" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="342" spans="1:3" x14ac:dyDescent="0.25">
@@ -12283,18 +12265,18 @@
         <v>987</v>
       </c>
       <c r="C361" t="s">
-        <v>988</v>
+        <v>282</v>
       </c>
     </row>
     <row r="362" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
+        <v>988</v>
+      </c>
+      <c r="B362" t="s">
         <v>989</v>
       </c>
-      <c r="B362" t="s">
+      <c r="C362" t="s">
         <v>990</v>
-      </c>
-      <c r="C362" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="363" spans="1:3" x14ac:dyDescent="0.25">
@@ -12302,21 +12284,21 @@
         <v>991</v>
       </c>
       <c r="B363" t="s">
-        <v>992</v>
+        <v>38</v>
       </c>
       <c r="C363" t="s">
-        <v>993</v>
+        <v>39</v>
       </c>
     </row>
     <row r="364" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
+        <v>992</v>
+      </c>
+      <c r="B364" t="s">
+        <v>993</v>
+      </c>
+      <c r="C364" t="s">
         <v>994</v>
-      </c>
-      <c r="B364" t="s">
-        <v>38</v>
-      </c>
-      <c r="C364" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="365" spans="1:3" x14ac:dyDescent="0.25">
@@ -12324,21 +12306,21 @@
         <v>995</v>
       </c>
       <c r="B365" t="s">
-        <v>996</v>
+        <v>993</v>
       </c>
       <c r="C365" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
     </row>
     <row r="366" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
+        <v>996</v>
+      </c>
+      <c r="B366" t="s">
+        <v>997</v>
+      </c>
+      <c r="C366" t="s">
         <v>998</v>
-      </c>
-      <c r="B366" t="s">
-        <v>996</v>
-      </c>
-      <c r="C366" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="367" spans="1:3" x14ac:dyDescent="0.25">
@@ -12632,29 +12614,29 @@
         <v>1077</v>
       </c>
       <c r="B393" t="s">
-        <v>1078</v>
+        <v>987</v>
       </c>
       <c r="C393" t="s">
-        <v>1079</v>
+        <v>282</v>
       </c>
     </row>
     <row r="394" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="B394" t="s">
-        <v>990</v>
+        <v>203</v>
       </c>
       <c r="C394" t="s">
-        <v>282</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="395" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B395" t="s">
         <v>1081</v>
-      </c>
-      <c r="B395" t="s">
-        <v>203</v>
       </c>
       <c r="C395" t="s">
         <v>1082</v>
@@ -12874,18 +12856,18 @@
         <v>1140</v>
       </c>
       <c r="B415" t="s">
+        <v>634</v>
+      </c>
+      <c r="C415" t="s">
         <v>1141</v>
-      </c>
-      <c r="C415" t="s">
-        <v>1142</v>
       </c>
     </row>
     <row r="416" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
+        <v>1142</v>
+      </c>
+      <c r="B416" t="s">
         <v>1143</v>
-      </c>
-      <c r="B416" t="s">
-        <v>634</v>
       </c>
       <c r="C416" t="s">
         <v>1144</v>
@@ -12972,7 +12954,7 @@
       <c r="A424" t="s">
         <v>1166</v>
       </c>
-      <c r="B424" t="s">
+      <c r="B424" s="1" t="s">
         <v>1167</v>
       </c>
       <c r="C424" t="s">
@@ -12983,7 +12965,7 @@
       <c r="A425" t="s">
         <v>1169</v>
       </c>
-      <c r="B425" s="1" t="s">
+      <c r="B425" t="s">
         <v>1170</v>
       </c>
       <c r="C425" t="s">
@@ -13104,7 +13086,7 @@
       <c r="A436" t="s">
         <v>1202</v>
       </c>
-      <c r="B436" t="s">
+      <c r="B436" s="1" t="s">
         <v>1203</v>
       </c>
       <c r="C436" t="s">
@@ -13115,7 +13097,7 @@
       <c r="A437" t="s">
         <v>1205</v>
       </c>
-      <c r="B437" s="1" t="s">
+      <c r="B437" t="s">
         <v>1206</v>
       </c>
       <c r="C437" t="s">
@@ -13192,7 +13174,7 @@
       <c r="A444" t="s">
         <v>1226</v>
       </c>
-      <c r="B444" t="s">
+      <c r="B444" s="1" t="s">
         <v>1227</v>
       </c>
       <c r="C444" t="s">
@@ -13203,7 +13185,7 @@
       <c r="A445" t="s">
         <v>1229</v>
       </c>
-      <c r="B445" s="1" t="s">
+      <c r="B445" t="s">
         <v>1230</v>
       </c>
       <c r="C445" t="s">
@@ -13401,7 +13383,7 @@
       <c r="A463" t="s">
         <v>1283</v>
       </c>
-      <c r="B463" t="s">
+      <c r="B463" s="1" t="s">
         <v>1284</v>
       </c>
       <c r="C463" t="s">
@@ -13423,7 +13405,7 @@
       <c r="A465" t="s">
         <v>1289</v>
       </c>
-      <c r="B465" s="1" t="s">
+      <c r="B465" t="s">
         <v>1290</v>
       </c>
       <c r="C465" t="s">
@@ -13544,7 +13526,7 @@
       <c r="A476" t="s">
         <v>1322</v>
       </c>
-      <c r="B476" t="s">
+      <c r="B476" s="1" t="s">
         <v>1323</v>
       </c>
       <c r="C476" t="s">
@@ -13566,7 +13548,7 @@
       <c r="A478" t="s">
         <v>1328</v>
       </c>
-      <c r="B478" s="1" t="s">
+      <c r="B478" t="s">
         <v>1329</v>
       </c>
       <c r="C478" t="s">
@@ -13586,24 +13568,24 @@
     </row>
     <row r="480" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>1334</v>
+        <v>1335</v>
       </c>
       <c r="B480" t="s">
-        <v>1335</v>
+        <v>1336</v>
       </c>
       <c r="C480" t="s">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="481" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>1337</v>
+        <v>1338</v>
       </c>
       <c r="B481" t="s">
-        <v>1338</v>
+        <v>1339</v>
       </c>
       <c r="C481" t="s">
-        <v>1339</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="482" spans="1:3" x14ac:dyDescent="0.25">
@@ -13622,32 +13604,32 @@
         <v>1344</v>
       </c>
       <c r="B483" t="s">
-        <v>1345</v>
+        <v>987</v>
       </c>
       <c r="C483" t="s">
-        <v>1346</v>
+        <v>282</v>
       </c>
     </row>
     <row r="484" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
+        <v>1345</v>
+      </c>
+      <c r="B484" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C484" t="s">
         <v>1347</v>
-      </c>
-      <c r="B484" t="s">
-        <v>1348</v>
-      </c>
-      <c r="C484" t="s">
-        <v>1349</v>
       </c>
     </row>
     <row r="485" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
+        <v>1348</v>
+      </c>
+      <c r="B485" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C485" t="s">
         <v>1350</v>
-      </c>
-      <c r="B485" t="s">
-        <v>990</v>
-      </c>
-      <c r="C485" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="486" spans="1:3" x14ac:dyDescent="0.25">
@@ -14219,48 +14201,48 @@
         <v>1505</v>
       </c>
       <c r="C537" t="s">
-        <v>1506</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" t="s">
+        <v>1506</v>
+      </c>
+      <c r="B538" t="s">
         <v>1507</v>
       </c>
-      <c r="B538" t="s">
+      <c r="C538" t="s">
         <v>1508</v>
-      </c>
-      <c r="C538" t="s">
-        <v>1509</v>
       </c>
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" t="s">
+        <v>1509</v>
+      </c>
+      <c r="B539" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C539" t="s">
         <v>1510</v>
-      </c>
-      <c r="B539" t="s">
-        <v>1511</v>
-      </c>
-      <c r="C539" t="s">
-        <v>1309</v>
       </c>
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" t="s">
+        <v>1511</v>
+      </c>
+      <c r="B540" t="s">
         <v>1512</v>
       </c>
-      <c r="B540" t="s">
+      <c r="C540" t="s">
         <v>1513</v>
-      </c>
-      <c r="C540" t="s">
-        <v>1514</v>
       </c>
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" t="s">
+        <v>1514</v>
+      </c>
+      <c r="B541" t="s">
         <v>1515</v>
-      </c>
-      <c r="B541" t="s">
-        <v>1499</v>
       </c>
       <c r="C541" t="s">
         <v>1516</v>
@@ -14689,29 +14671,29 @@
         <v>1631</v>
       </c>
       <c r="B580" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C580" t="s">
         <v>1632</v>
-      </c>
-      <c r="C580" t="s">
-        <v>1633</v>
       </c>
     </row>
     <row r="581" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A581" t="s">
+        <v>1633</v>
+      </c>
+      <c r="B581" t="s">
         <v>1634</v>
       </c>
-      <c r="B581" t="s">
+      <c r="C581" t="s">
         <v>1635</v>
-      </c>
-      <c r="C581" t="s">
-        <v>1636</v>
       </c>
     </row>
     <row r="582" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A582" t="s">
+        <v>1636</v>
+      </c>
+      <c r="B582" t="s">
         <v>1637</v>
-      </c>
-      <c r="B582" t="s">
-        <v>1499</v>
       </c>
       <c r="C582" t="s">
         <v>1638</v>
@@ -15165,29 +15147,29 @@
         <v>1760</v>
       </c>
       <c r="C623" t="s">
-        <v>1761</v>
+        <v>614</v>
       </c>
     </row>
     <row r="624" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A624" t="s">
+        <v>1761</v>
+      </c>
+      <c r="B624" t="s">
         <v>1762</v>
       </c>
-      <c r="B624" t="s">
+      <c r="C624" t="s">
         <v>1763</v>
-      </c>
-      <c r="C624" t="s">
-        <v>1764</v>
       </c>
     </row>
     <row r="625" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A625" t="s">
+        <v>1764</v>
+      </c>
+      <c r="B625" t="s">
         <v>1765</v>
       </c>
-      <c r="B625" t="s">
+      <c r="C625" t="s">
         <v>1766</v>
-      </c>
-      <c r="C625" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="626" spans="1:3" x14ac:dyDescent="0.25">
@@ -15583,29 +15565,29 @@
         <v>1873</v>
       </c>
       <c r="C661" t="s">
-        <v>1874</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="662" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A662" t="s">
+        <v>1874</v>
+      </c>
+      <c r="B662" t="s">
         <v>1875</v>
       </c>
-      <c r="B662" t="s">
+      <c r="C662" t="s">
         <v>1876</v>
-      </c>
-      <c r="C662" t="s">
-        <v>1877</v>
       </c>
     </row>
     <row r="663" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A663" t="s">
+        <v>1877</v>
+      </c>
+      <c r="B663" t="s">
         <v>1878</v>
       </c>
-      <c r="B663" t="s">
+      <c r="C663" t="s">
         <v>1879</v>
-      </c>
-      <c r="C663" t="s">
-        <v>1192</v>
       </c>
     </row>
     <row r="664" spans="1:3" x14ac:dyDescent="0.25">
@@ -15803,29 +15785,29 @@
         <v>1932</v>
       </c>
       <c r="C681" t="s">
-        <v>1933</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="682" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A682" t="s">
+        <v>1933</v>
+      </c>
+      <c r="B682" t="s">
         <v>1934</v>
       </c>
-      <c r="B682" t="s">
+      <c r="C682" t="s">
         <v>1935</v>
-      </c>
-      <c r="C682" t="s">
-        <v>1936</v>
       </c>
     </row>
     <row r="683" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A683" t="s">
+        <v>1936</v>
+      </c>
+      <c r="B683" t="s">
         <v>1937</v>
       </c>
-      <c r="B683" t="s">
+      <c r="C683" t="s">
         <v>1938</v>
-      </c>
-      <c r="C683" t="s">
-        <v>1392</v>
       </c>
     </row>
     <row r="684" spans="1:3" x14ac:dyDescent="0.25">
@@ -16595,29 +16577,29 @@
         <v>2147</v>
       </c>
       <c r="C753" t="s">
-        <v>2148</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="754" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A754" t="s">
+        <v>2148</v>
+      </c>
+      <c r="B754" t="s">
         <v>2149</v>
       </c>
-      <c r="B754" t="s">
+      <c r="C754" t="s">
         <v>2150</v>
-      </c>
-      <c r="C754" t="s">
-        <v>2151</v>
       </c>
     </row>
     <row r="755" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A755" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B755" t="s">
         <v>2152</v>
       </c>
-      <c r="B755" t="s">
+      <c r="C755" t="s">
         <v>2153</v>
-      </c>
-      <c r="C755" t="s">
-        <v>1340</v>
       </c>
     </row>
     <row r="756" spans="1:3" x14ac:dyDescent="0.25">
@@ -16683,29 +16665,29 @@
         <v>2170</v>
       </c>
       <c r="C761" t="s">
-        <v>2171</v>
+        <v>294</v>
       </c>
     </row>
     <row r="762" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A762" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B762" t="s">
         <v>2172</v>
       </c>
-      <c r="B762" t="s">
+      <c r="C762" t="s">
         <v>2173</v>
-      </c>
-      <c r="C762" t="s">
-        <v>2174</v>
       </c>
     </row>
     <row r="763" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A763" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B763" t="s">
         <v>2175</v>
       </c>
-      <c r="B763" t="s">
+      <c r="C763" t="s">
         <v>2176</v>
-      </c>
-      <c r="C763" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="764" spans="1:3" x14ac:dyDescent="0.25">
@@ -16716,29 +16698,29 @@
         <v>2178</v>
       </c>
       <c r="C764" t="s">
-        <v>2179</v>
+        <v>1519</v>
       </c>
     </row>
     <row r="765" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A765" t="s">
+        <v>2179</v>
+      </c>
+      <c r="B765" t="s">
         <v>2180</v>
       </c>
-      <c r="B765" t="s">
+      <c r="C765" t="s">
         <v>2181</v>
-      </c>
-      <c r="C765" t="s">
-        <v>2182</v>
       </c>
     </row>
     <row r="766" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A766" t="s">
+        <v>2182</v>
+      </c>
+      <c r="B766" t="s">
         <v>2183</v>
       </c>
-      <c r="B766" t="s">
+      <c r="C766" t="s">
         <v>2184</v>
-      </c>
-      <c r="C766" t="s">
-        <v>1525</v>
       </c>
     </row>
     <row r="767" spans="1:3" x14ac:dyDescent="0.25">
@@ -16848,29 +16830,29 @@
         <v>2213</v>
       </c>
       <c r="C776" t="s">
-        <v>2214</v>
+        <v>497</v>
       </c>
     </row>
     <row r="777" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A777" t="s">
+        <v>2214</v>
+      </c>
+      <c r="B777" t="s">
         <v>2215</v>
       </c>
-      <c r="B777" t="s">
+      <c r="C777" t="s">
         <v>2216</v>
-      </c>
-      <c r="C777" t="s">
-        <v>2217</v>
       </c>
     </row>
     <row r="778" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A778" t="s">
+        <v>2217</v>
+      </c>
+      <c r="B778" t="s">
         <v>2218</v>
       </c>
-      <c r="B778" t="s">
+      <c r="C778" t="s">
         <v>2219</v>
-      </c>
-      <c r="C778" t="s">
-        <v>497</v>
       </c>
     </row>
     <row r="779" spans="1:3" x14ac:dyDescent="0.25">
@@ -17739,29 +17721,29 @@
         <v>2455</v>
       </c>
       <c r="C857" t="s">
-        <v>2456</v>
+        <v>2438</v>
       </c>
     </row>
     <row r="858" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A858" t="s">
+        <v>2456</v>
+      </c>
+      <c r="B858" t="s">
         <v>2457</v>
       </c>
-      <c r="B858" t="s">
+      <c r="C858" t="s">
         <v>2458</v>
-      </c>
-      <c r="C858" t="s">
-        <v>2459</v>
       </c>
     </row>
     <row r="859" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A859" t="s">
+        <v>2459</v>
+      </c>
+      <c r="B859" t="s">
         <v>2460</v>
       </c>
-      <c r="B859" t="s">
+      <c r="C859" t="s">
         <v>2461</v>
-      </c>
-      <c r="C859" t="s">
-        <v>2444</v>
       </c>
     </row>
     <row r="860" spans="1:3" x14ac:dyDescent="0.25">
@@ -18334,28 +18316,6 @@
       </c>
       <c r="C911" t="s">
         <v>2617</v>
-      </c>
-    </row>
-    <row r="912" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A912" t="s">
-        <v>2618</v>
-      </c>
-      <c r="B912" t="s">
-        <v>2619</v>
-      </c>
-      <c r="C912" t="s">
-        <v>2620</v>
-      </c>
-    </row>
-    <row r="913" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A913" t="s">
-        <v>2621</v>
-      </c>
-      <c r="B913" t="s">
-        <v>2622</v>
-      </c>
-      <c r="C913" t="s">
-        <v>2623</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove false positive (#5522)
</commit_message>
<xml_diff>
--- a/add-in-ids/add-ins-using-exchange-tokens.xlsx
+++ b/add-in-ids/add-ins-using-exchange-tokens.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28619"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28717"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B9BDEF2-8F23-4ECC-BD34-7BD727B64A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FEC815D-DD99-44A2-8C08-999040041229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19395" yWindow="465" windowWidth="18180" windowHeight="14130" xr2:uid="{8FF931F1-CAD9-4954-9038-88E82260DB46}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{8FF931F1-CAD9-4954-9038-88E82260DB46}"/>
   </bookViews>
   <sheets>
     <sheet name="Add-ins list" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2729" uniqueCount="2619">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2726" uniqueCount="2616">
   <si>
     <t>AssetID</t>
   </si>
@@ -6709,15 +6709,6 @@
   </si>
   <si>
     <t>Awardco</t>
-  </si>
-  <si>
-    <t>wa200004958</t>
-  </si>
-  <si>
-    <t>bb2dab9e-522f-4e44-a001-2457d335e721</t>
-  </si>
-  <si>
-    <t>Showpad for Outlook</t>
   </si>
   <si>
     <t>wa200004960</t>
@@ -7972,8 +7963,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}" name="Table1" displayName="Table1" ref="A1:C911" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:C911" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}" name="Table1" displayName="Table1" ref="A1:C910" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:C910" xr:uid="{CD6B8178-56C6-442C-A6BF-7C2D1F869861}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{39B649A1-0CDF-46AA-A276-6F4F89255D96}" name="AssetID"/>
     <tableColumn id="2" xr3:uid="{C79A1EFF-47FF-488B-A562-E9848648C952}" name="AppId"/>
@@ -8300,7 +8291,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3293B4AA-89CE-4E6A-9112-DA5B905DDA88}">
-  <dimension ref="A1:C911"/>
+  <dimension ref="A1:C910"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" customWidth="1"/>
@@ -8314,7 +8305,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>2618</v>
+        <v>2615</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -17710,18 +17701,18 @@
         <v>2452</v>
       </c>
       <c r="C856" t="s">
-        <v>2453</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="857" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A857" t="s">
+        <v>2453</v>
+      </c>
+      <c r="B857" t="s">
         <v>2454</v>
       </c>
-      <c r="B857" t="s">
+      <c r="C857" t="s">
         <v>2455</v>
-      </c>
-      <c r="C857" t="s">
-        <v>2438</v>
       </c>
     </row>
     <row r="858" spans="1:3" x14ac:dyDescent="0.25">
@@ -18305,17 +18296,6 @@
       </c>
       <c r="C910" t="s">
         <v>2614</v>
-      </c>
-    </row>
-    <row r="911" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A911" t="s">
-        <v>2615</v>
-      </c>
-      <c r="B911" t="s">
-        <v>2616</v>
-      </c>
-      <c r="C911" t="s">
-        <v>2617</v>
       </c>
     </row>
   </sheetData>

</xml_diff>